<commit_message>
docs: T11 — LLM_API명세서.xlsx 전면 동기화 (14 → 24행, openapi 전수 일치)
- API 명세서 시트: LLM-015~024 10행 신설(신규 채번 — Notion 대조 후 확정),
  LLM-005 전면 개정(통합 요청 11필드·policy_params 제거·9종·언더바·0 허용·
  rule_file_ref=파일명), LLM-004 dead 케이스, LLM-006 파일 회칙 지원(구
  '텍스트만 지원' 폐기), 검증: URL+Method 집합 == openapi 24오퍼레이션
- AI 마법사 연동 시트: 2단계 개편(금액 1칸·경계 이상·배수 계산 폐기·0=전건
  확인), 카테고리 전역 9종, escalation_threshold 부재(8/6 정정) 3곳
- 콜백·내부API 시트: CB-001 11키(제거 4필드 정리)·auditor 4종(evidence),
  BE-001 category null, BE-002 컬럼 부재, BE-004 경로 확정+토큰 잠금 권장,
  BE-005 content-type 분기·팀당 1개, BE-006 언더바 표기
- 상태코드 시트: 동기/비동기 목록에 신규 ID 반영
</commit_message>
<xml_diff>
--- a/docs/LLM_API명세서.xlsx
+++ b/docs/LLM_API명세서.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -671,7 +671,8 @@
         <is>
           <t>콜백 유실 대비 폴링 fallback. job_id·external_job_id 어느 쪽으로도 조회 가능.
 status: queued / running / succeeded / failed / dead(재시도 소진)
-succeeded면 result에 심사 결과(verdict·reasons·opinions)가 담김</t>
+succeeded면 result에 심사 결과(verdict·reasons·opinions)가 담김
+dead면 result = {"error": "&lt;예외 클래스명&gt;", "message": "&lt;실패 사유&gt;"} — 화면에는 message만 쓰세요 (회칙 파싱 실패 DocumentParseError 계열만 원문이고, 그 외 예외는 정형 문구입니다)</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -701,7 +702,7 @@
       <c r="C6" s="3" t="inlineStr">
         <is>
           <t>모임 생성
-마법사 1·3단계</t>
+마법사 1~3단계</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -716,22 +717,22 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>team_type*,
+          <t>team_id*,
+team_type*,
 team_name*,
 initial_budget*,
 member_count,
 description,
-dues</t>
+dues,
+force_escalation_amount*,
+rule_source*,
+rule_text (manual 필수),
+rule_file_ref (file 필수)</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
           <t>rules[],
-policy_params: {
-  auto_approve_limit,
-  force_escalation_amount,
-  confidence_threshold
-},
 recommended_categories[],
 notes</t>
         </is>
@@ -748,11 +749,14 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>동기 응답(마법사 UX). 회칙 조항 + 에이전트 정책 파라미터 + 유형별 카테고리 6개 추천.
-모임 소개(description)가 있으면 AI가 그 모임 특색 조항을 최대 3개 추가.
-회비(dues)를 보내주시면 회비 조항이 1개 더 붙습니다 — null·0은 "없음"으로 처리.
-한도 수치는 코드가 계산 — LLM이 지어내지 않음. force_escalation_amount = auto_approve_limit × 4 (마법사 2단계 구간표 기준)
-※ 이 API는 요청·응답 모두 snake_case입니다 (camelCase는 LLM-003 심사 요청과 콜백뿐).</t>
+          <t>동기 응답(마법사 UX). 마법사 1~3단계 통합 요청 — 2026-08-05 전면 개정.
+· rules는 rule_source=ai일 때만 채움(그 외 빈 배열) — 문자열 배열, 항목당 완결된 조항 한 문장
+· policy_params 응답 제거 — 승인 정책은 사용자 입력 기준 금액이 원천(AI가 제안하지 않음)
+· recommended_categories는 전역 9종 고정 — 구판의 모임 유형별 추천은 폐기
+· team_type은 백엔드 ENUM 언더바 표기 그대로(동아리_학생회 등 5종) — 저희가 내부 표기로 변환
+· force_escalation_amount 0 = 전건 관리자 확인('모든 지출 직접 확인' 토글, 8/6 확정) · 음수만 422
+· rule_source: file / manual / ai / skip · file이면 rule_file_ref에 저장된 파일명(예: bd345b5a-….pdf)
+· dues는 null·0 둘 다 '없음' · 요청·응답 모두 snake_case (camelCase는 LLM-003 심사 요청과 콜백뿐)</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -819,8 +823,8 @@
 ※ 이 호출이 없으면 저희는 계속 옛 회칙으로 심사하게 됩니다
 ※ 마법사 3단계에서 회칙을 등록(API-031)하신 직후에도 호출이 필요합니다
 ※ 이 API는 요청·응답 모두 snake_case입니다 (camelCase는 LLM-003 심사 요청과 콜백뿐).
-※ 응답 job_id를 LLM-004로 조회하면 인덱싱 완료(succeeded)를 확인하실 수 있습니다 — 마법사 4단계 policySyncStatus=READY 판정에 쓰세요.
-※ 회칙 원문은 텍스트만 지원합니다 — PDF·이미지 파서는 아직 없습니다. 마법사 3단계 파일 업로드분은 텍스트로 추출해 BE-005로 주세요.</t>
+※ 응답 job_id를 LLM-004로 조회하면 인덱싱 완료(succeeded)를 확인하실 수 있습니다 — 마법사 4단계 policySyncStatus=READY 판정에 쓰세요(LLM-022로도 확인 가능).
+※ 회칙이 파일(PDF·Word)로 등록된 팀도 이 계약 그대로입니다 — BE-005가 원본 파일을 반환하면 저희가 파싱합니다(2026-08-06 확장). 텍스트 추출은 필요 없습니다</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -894,558 +898,1173 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>■ 리포트·제안  (잡 방식 — 202 응답 후 LLM-004로 폴링)</t>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>LLM-018</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>카테고리 목록 조회</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>지출 등록 ·
+마법사 1단계</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>/v1/categories</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>categories[] (9종),
+fallback,
+version</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>전역 고정 9종 — LLM-005 응답 recommended_categories와 같은 목록.
+확정 9종: 회의 · IT_인프라 · 행사_활동 · 장소_대관 · 교육 · 식비 · 교통 · 비품 · 기타</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
+          <t>LLM-019</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>저장된 회칙 초안 조회</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>회칙·정책 관리</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>/v1/policy-proposals</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>?team_id*</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>(저장된 초안)
+또는 null</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>401, 422</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>마법사 회칙 초안(rule_draft) 전용 조회 — 없으면 404가 아니라 200 + null.
+관리자 제안함 목록(LLM-015)과는 별개 자원입니다</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>LLM-020</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>승인 정책 적용 상태 조회</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>마법사 2단계
+(저장 직후 확인)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>/v1/policy-params/status</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>?organization_id*</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>available,
+auto_approve,
+auto_approve_limit,
+force_escalation_amount,
+effective_auto_approve_limit,
+auto_approved_up_to,
+summary,
+team_id</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>401, 422</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>2단계 저장값이 실제 심사에 어떻게 적용되는지 확인 — summary를 화면에 그대로 띄우면 됩니다.
+escalation_threshold 컬럼 부재(8/6 정정)라 force_escalation_amount는 항상 auto_approve_limit과 같습니다</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>LLM-021</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>회칙 초안 생성·저장</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>회칙·정책 관리</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>/v1/policy-proposals</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>(LLM-005와 같은 필드),
+regenerate</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>proposal_id,
+team_id,
+status,
+reused,
+draft{rules[],
+  recommended_categories[],
+  notes}</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>401, 422, 500</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>LLM-005의 저장형 — 초안을 만들어 proposals에 남긴다. 미결정 초안이 있으면 재사용(reused=true)하고, 관리자가 '다시 생성'을 눌렀을 때만 regenerate=true로 새로 만든다.
+rule_source는 ai로 고정(생략 가능)</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>LLM-022</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>회칙 인덱싱 상태 조회</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>마법사 4단계</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>/v1/context/status</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>?team_id*</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>team_id,
+indexed,
+chunk_count,
+version,
+indexed_at</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>401, 422</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>LLM-006 인덱싱이 끝났는지 확인 — policySyncStatus=READY 판정 보조(LLM-004 폴링의 대안)</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>■ 리포트·제안·대시보드 — LLM-008~011·016은 202 잡 접수(LLM-004 폴링) · LLM-015·017은 동기 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>LLM-008</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>정산 리포트 생성</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>정산</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>/v1/reports/summary</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>team_id*,
 period*</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>job_id,
 external_job_id,
 status</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>401, 422</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>202</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>기간 지출 집계 + AI 요약 + 예산 활용 추천.
 수치는 코드가 계산하고 검산을 통과한 것만 반환</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="K15" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>LLM-009</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>주간 브리핑 생성</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>대시보드</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>/v1/digests</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>team_id*,
 week_of*</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>job_id,
 external_job_id,
 status</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>401, 422</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>202</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>주간 자동처리 현황 · 예산 소진 전망 · 이상 징후 + 총무 코멘트</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K16" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>LLM-010</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>인수인계 브리핑 생성</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>총무 교체</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>/v1/briefings</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>team_id*</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>job_id,
 external_job_id,
 status</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>401, 422</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>202</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>총무 교체 시 인계 사항 정리</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="K17" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>LLM-011</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>회칙 개정 제안 생성</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>회칙 관리</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>/v1/proposals/rule-amendment</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>team_id*</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>job_id,
 external_job_id,
 status</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>401, 422</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>202</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>관리자가 같은 패턴으로 3회 이상 개입한 건을 찾아 회칙 공백을 진단하고 개정 문안 제안</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K18" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>LLM-012</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>제안 수락/기각</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>회칙 관리</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>/v1/proposals/{proposal_id}</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>PATCH</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>status*,
 decided_by*</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>(갱신 결과)</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>401, 404, 409, 422</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="J19" s="3" t="inlineStr">
         <is>
           <t>status: accepted / dismissed
 이미 결정된 건을 다시 결정하면 409</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="K19" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>■ 헬스체크·내부 평가</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>LLM-015</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>AI 제안 목록 조회</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>관리자 제안함</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>/v1/proposals</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>?team_id*
+&amp;type &amp;status (선택)</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>[{id, team_id, type,
+  payload, status,
+  decided_by,
+  created_at, decided_at}]</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>401, 422</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>AI가 올린 제안 목록 — 없으면 빈 배열(404 아님).
+type 미지정 시 마법사 회칙 초안(rule_draft)은 제외 — 그쪽은 LLM-019가 다루는 별개 자원이라 중복 노출을 막기 위함. type=rule_draft를 명시하면 포함</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>LLM-016</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>예산 관리 AI 메시지 생성</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>예산 관리</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>/v1/proposals/budget</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>team_id*,
+period (선택 —
+미지정 시 당월)</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>job_id,
+external_job_id,
+status</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>401, 422</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>202</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>202 잡 접수 — 결과는 LLM-004 폴링 또는 GET /v1/proposals?type=budget.
+payload는 Figma 확정 3블록(category_analysis · budget_status_analysis · recommendation) + figures + verified.
+★ verified=false여도 안전 문장으로 교체 저장되므로 3블록은 항상 그대로 화면 표시 가능 — LLM-017과 반대 규칙</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>LLM-017</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>대시보드 AI 요약 생성</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>대시보드</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>/v1/dashboard/summary</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>team_id*,
+period (선택 —
+미지정 시 당월)</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>figures{...},
+message,
+verified</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>401, 422</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>동기 응답(202 아님).
+집계 3종 확정(8/6 회신): 전월 대비 증감 최대 카테고리·증감률 / 전체 예산 사용률 / 잔여 예산·남은 기간 코멘트.
+★ verified=false면 message를 화면에 띄우지 말거나 '확인 필요' 표시 — LLM-016과 반대 규칙</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>■ 헬스체크·내부 전용 — LLM-013·014·023·024는 연동 대상 아님</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>LLM-001</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>라이브니스</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>(인프라)</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>/healthz</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H24" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="J24" s="3" t="inlineStr">
         <is>
           <t>프로세스 생존 확인</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="K24" s="3" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>LLM-002</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>레디니스</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>(인프라)</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>/readyz</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>?deep=true (선택)</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>status,
 checks</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>503</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="I25" s="3" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="J25" s="3" t="inlineStr">
         <is>
           <t>DB·LLM 준비 상태 점검. deep=true면 OpenAI 도달성까지 확인</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="K25" s="3" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>LLM-013</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>골든셋 평가 결과</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>(내부)</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>/v1/eval/golden</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>(평가 지표)</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>401</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr">
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>LLM팀 내부 검증용 — 연동 대상 아님</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="K26" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>LLM-014</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>생성물 평가 결과</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>(내부)</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>/v1/eval/writers</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>(평가 지표)</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>401</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr">
+      <c r="J27" s="3" t="inlineStr">
         <is>
           <t>LLM팀 내부 검증용 — 연동 대상 아님</t>
         </is>
       </c>
-      <c r="K19" s="3" t="inlineStr">
+      <c r="K27" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>* 표시 = 필수 필드 · 모든 요청에 Authorization: Bearer &lt;SERVICE_TOKEN&gt; 필요(인증 N 제외) · 값 출처: docs/openapi.json (코드 자동 생성)</t>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>LLM-023</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>심사 스트림 데모</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>(내부)</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>/v1/reviews/stream</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>(LLM-003과 동일)</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>SSE 스트림</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>401, 422</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>LLM팀 내부 데모·관측 전용(실시간 진행 표시) — 연동 대상 아님</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>LLM-024</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>심사 개입 결정</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>(내부)</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>/v1/reviews/{job_id}/decision</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>decision*,
+reason</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>(재개 결과)</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>401, 422</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>LLM팀 내부 데모 전용(관리자 개입 시연) — 연동 대상 아님</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>* 표시 = 필수 필드 · 모든 요청에 Authorization: Bearer &lt;SERVICE_TOKEN&gt; 필요(인증 N 제외) · 값 출처: docs/openapi.json (코드 자동 생성) · LLM-015~024 행 신설 + LLM-004~006 개정: 2026-08-06 (T11)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A15:K15"/>
-    <mergeCell ref="A9:K9"/>
+    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="A23:K23"/>
     <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1547,7 +2166,8 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>LLM 호출·프로세스 생성 없음. 한 트랜잭션으로 teams + team_members(인증 사용자 ADMIN) + budgets + 기본 team_settings(autoApprove=false, escalationThreshold=200000)를 생성하는 안입니다 (회신요청 16번)</t>
+          <t>LLM 호출·프로세스 생성 없음. 한 트랜잭션으로 teams + team_members(인증 사용자 ADMIN) + budgets + 기본 team_settings(autoApprove=false)를 생성하는 안입니다 (회신요청 16번).
+※ escalation_threshold 컬럼은 존재하지 않습니다(8/6 백엔드 정정) — 저장은 auto_approve_limit 하나</t>
         </is>
       </c>
     </row>
@@ -1584,8 +2204,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>★ 신규 반영 — 저희 쪽 필드는 이미 열어 뒀습니다. 안 보내주셔도 지금처럼 동작합니다.
-null / 0 중 어느 쪽으로 보내실지만 알려주세요 (회신요청 15번 ①)</t>
+          <t>null·0 둘 다 '없음'으로 동작합니다 — 어느 쪽을 보내셔도 무방하고, 안 보내셔도 지금처럼 동작합니다</t>
         </is>
       </c>
     </row>
@@ -1617,12 +2236,12 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>모임 유형별 6종</t>
+          <t>전역 고정 9종</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>DB category ENUM 7종과 겹치는 값이 0건입니다 — ENUM 확장 요청 중 (회신요청 3번)</t>
+          <t>✅ ENUM 9종 확장 확정(8/5) + expenses.category nullable 전환 완료(8/6) — 등록 시 null 저장, 콜백 suggestedCategory로 채움</t>
         </is>
       </c>
     </row>
@@ -1644,22 +2263,24 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>LLM-005 응답 policy_params.force_escalation_amount</t>
+          <t>LLM-005 요청 force_escalation_amount</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>LLM → BE → FE</t>
+          <t>FE → BE → LLM</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>auto_approve_limit × 4</t>
+          <t>사용자 입력 금액 1칸
+(최소 5만원 — 화면 강제)</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>★ 화면의 20만원 기준에 맞춰 배수를 6 → 4로 바꿨습니다</t>
+          <t>★ 2026-08-05 개편 — 금액 칸 2개 → 1개('관리자 승인 필수 금액'), 경계 '이상'. AI 추천(배수 계산)은 폐기 — 사용자 입력이 원천이고 저희는 제안하지 않습니다.
+0 = 전건 관리자 확인('모든 지출 직접 확인' 토글 켬, 8/6 확정)</t>
         </is>
       </c>
     </row>
@@ -1676,28 +2297,28 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>소액 / 중간 / 고액 구간표</t>
+          <t>심사 구간 안내 (2구간)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>LLM-005 응답 policy_params</t>
+          <t>(화면 자체 표시 — LLM 호출 없음)</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>LLM → BE → FE</t>
+          <t>FE</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>auto_approve_limit,
-force_escalation_amount</t>
+          <t>기준 금액 미만 = AI 자동 심사
+기준 금액 이상 = 관리자 확인</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>제안 구간: amount &lt; autoApproveLimit / autoApproveLimit 이상~escalationThreshold 미만 / escalationThreshold 이상. 중간 구간은 검사 결과와 AI 확신도에 따라 자동 또는 관리자 검토 (회신요청 15번 ⑤·16번)</t>
+          <t>구 3구간(소액/중간/고액)은 2026-08-05 개편으로 2구간이 됐습니다. 저장값이 심사에 어떻게 적용되는지는 LLM-020(GET /v1/policy-params/status)로 확인</t>
         </is>
       </c>
     </row>
@@ -1731,13 +2352,13 @@
         <is>
           <t>membershipFee,
 autoApprove,
-autoApproveLimit,
-escalationThreshold</t>
+autoApproveLimit</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>API-028·029에 네 필드를 포함하고, policySyncStatus != READY이면 내부 Agent API의 유효 auto_approve는 false로 내려 자동 승인을 차단하는 안입니다</t>
+          <t>API-028·029에 세 필드를 포함하고, policySyncStatus != READY이면 내부 Agent API의 유효 auto_approve는 false로 내려 자동 승인을 차단하는 안입니다.
+※ escalation_threshold 컬럼 부재(8/6 정정). 토글 켬 = autoApprove=false · autoApproveLimit=null 저장 — LLM-005 요청에는 0으로 전달</t>
         </is>
       </c>
     </row>
@@ -1813,7 +2434,8 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>정책·버전과 Outbox 이벤트를 같은 DB 트랜잭션으로 저장한 뒤, 커밋 후 LLM-006을 호출합니다. 인덱싱 중에는 policySyncStatus=PENDING</t>
+          <t>정책·버전과 Outbox 이벤트를 같은 DB 트랜잭션으로 저장한 뒤, 커밋 후 LLM-006을 호출합니다. 인덱싱 중에는 policySyncStatus=PENDING.
+※ 파일(PDF·Word)은 그대로 저장하시면 됩니다 — BE-005가 원본을 반환하면 저희가 파싱합니다(8/6 확장). LLM-005 요청 rule_file_ref에는 저장된 파일명을 넣어 주세요</t>
         </is>
       </c>
     </row>
@@ -2026,8 +2648,7 @@
 processedBy, confidence,
 opinions[], mismatch[],
 reasons{requester, admin},
-modelVersion, promptVersion,
-costUsd, latencyMs, dryRun</t>
+dryRun</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -2049,7 +2670,10 @@
         <is>
           <t>심사 완료 시 LLM 서버가 발신. 최대 3회 재시도(지수 백오프 1s→2s), 타임아웃 10초.
 3회 실패해도 잡은 죽지 않고 LLM-004 폴링이 안전망 → 같은 콜백이 중복 도착할 수 있습니다.
-⚠ 파서 주의: opinions[].similar_cases만 snake_case / mismatch[].claimed·receipt는 문자열</t>
+⚠ 파서 주의: opinions[].similar_cases만 snake_case / mismatch[].claimed·receipt는 문자열
+⚠ 최상위 키는 11개 — 구판의 modelVersion·promptVersion·costUsd·latencyMs 4개는 제거(2026-08-03). 전환기에 더 실려 올 수 있으니 모르는 필드는 무시하는 파서로 만들어 주세요.
+opinions[].auditor는 4종: rule / budget / precedent / evidence — evidence(증빙 심사관)는 영수증-청구 대조 소견으로 지출 상세 'AI 심사결과' 표시용이며 판정 권한이 없습니다.
+suggestedCategory는 전역 9종 값으로 갑니다</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -2114,7 +2738,8 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>pull 모델의 핵심 — 심사할 지출의 내용. category가 빈 값이면 AI가 자동 분류.
+          <t>pull 모델의 핵심 — 심사할 지출의 내용.
+✅ category는 null로 주세요(8/6 확정 — 등록 시 null 저장). 항상 AI가 분류해 콜백 suggestedCategory로 돌려드립니다. 값이 채워져 오면 경고 로그 후 AI 분류로 덮습니다.
 조회 실패 시 재시도 후 fail-safe 에스컬레이션(자동 승인으로 이어지지 않음)</t>
         </is>
       </c>
@@ -2158,8 +2783,7 @@
       <c r="G6" s="3" t="inlineStr">
         <is>
           <t>auto_approve,
-auto_approve_limit,
-escalation_threshold</t>
+auto_approve_limit</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -2175,8 +2799,8 @@
       <c r="J6" s="3" t="inlineStr">
         <is>
           <t>자동승인 권한·한도 — 가드레일 0번 규칙(최상위 게이트).
-escalation_threshold는 금액으로 확정 — 저희 force_escalation_amount와 1:1입니다.
-※ 기본값을 200,000원으로 맞추실지 회신 부탁드립니다 (저희 코드 기본값은 200,000원으로 내렸습니다 — 회신요청 15번 ④)</t>
+✅ escalation_threshold 컬럼은 존재하지 않습니다(8/6 백엔드 정정 — auto_approve_limit 하나만).
+auto_approve_limit null = 전건 관리자 확인(안전 방향) · 경계는 '이상'(한도 5만이면 5만부터 관리자 확인)</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -2262,7 +2886,8 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>요청의 receiptPath 경로</t>
+          <t>/api/files/{fileName}
+(요청의 receiptPath로 전달)</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -2295,7 +2920,8 @@
         <is>
           <t>Vision OCR로 금액·날짜 추출 → 신청 금액과 불일치 시 무조건 보류.
 판독 실패해도 심사는 멈추지 않고 에스컬레이션.
-※ 값 형식 미확정 — 내부 경로/서명 URL/파일 ID 중 무엇인지 (회신요청 1번)</t>
+✅ 경로 확정(8/6) — 기존 GET /api/files/{fileName} 그대로(지출 상세 receiptFileUrl 형태).
+★ Agent 토큰 잠금 권장 — 저희는 항상 토큰을 보내므로 막아도 무영향(프론트 사용 여부만 확인 필요)</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -2338,7 +2964,9 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>text (원문 전체)</t>
+          <t>JSON { text } 또는
+파일 원본 바이트
+(Content-Type로 판별)</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -2353,8 +2981,9 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>LLM-006(회칙 변경 알림) 수신 직후 호출해 청킹·임베딩·재인덱싱합니다.
-원문 무수정 전달 필요</t>
+          <t>LLM-006(회칙 변경 알림) 수신 직후 호출해 청킹·임베딩·재인덱싱합니다. 원문 무수정 전달 필요.
+✅ 판별 규칙 확정(8/6): 텍스트 = application/json + {"text"} / 파일 = 원본 MIME(pdf·docx) + 바이트 + Content-Disposition filename. base64·URL로 감싸지 않습니다.
+회칙은 팀당 1개(덮어쓰기) — version 파라미터는 사실상 항상 최신 1건(무시하셔도 됩니다)</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -2412,7 +3041,7 @@
       <c r="J10" s="3" t="inlineStr">
         <is>
           <t>모임 유형별 카테고리 카탈로그 선택에 사용.
-유형 5종: 동아리/학생회 · 스터디 · 친목 · 동호회 · 회사 (문자열 정확히 일치 필요)</t>
+✅ 유형 5종 — 백엔드 ENUM 언더바 표기 그대로(8/6 확정): 동아리_학생회 · 스터디 · 친목 · 동호회 · 회사. 저희가 내부 표기로 변환합니다(첫 값의 정확한 표기는 재확인 중)</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -2599,7 +3228,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>동기 응답 — 잡 조회(LLM-004) · 회칙 초안(LLM-005) · 제안 결정(LLM-012)</t>
+          <t>동기 응답 — 잡 조회(LLM-004) · 마법사 통합 요청(LLM-005) · 제안 결정(LLM-012) · 제안 목록(LLM-015) · 대시보드 요약(LLM-017) · 조회 4종(LLM-018 카테고리 · 019 초안 · 020 정책상태 · 022 인덱싱상태) · 초안 저장(LLM-021)</t>
         </is>
       </c>
     </row>
@@ -2633,7 +3262,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>비동기 잡 등록 — 심사(LLM-003) · 리포트·제안(LLM-008~011).
+          <t>비동기 잡 등록 — 심사(LLM-003) · 리포트·제안(LLM-008~011) · 예산 메시지(LLM-016).
 결과는 콜백 또는 LLM-004 폴링으로 받습니다</t>
         </is>
       </c>

</xml_diff>